<commit_message>
fix: Phase 6.9 review patches (Sprint 2) — mangle xlsx port codes to bad-shape
Spec §6.1.2 was explicit: refresh the fixture's port codes to bad-shape
values that R1 will catch (e.g., 'zz', 'USXX1', 'USX@1'). Codex's Phase
6.9 implementation left this incomplete (Critique #3 acknowledged the
gap but deferred to V8). Without the mangling, ZZZZZ and QQQQQ pass the
UN/LOCODE shape regex ^[A-Z]{2}[A-Z0-9]{3}$, so R1 would not fire and
the integration test
test_broken_impossible_port_codes_rejects_with_port_unknown_unlocode
would fail in V8 F.4.

Change: row 4 col A (origin)      ZZZZZ -> ZZ@ZZ
        row 6 col B (destination) QQQQQ -> QQ@QQ

Both new codes contain '@' (non A-Z, non 0-9), failing the regex
deterministically. Validity columns (2026-06-01 / 2026-12-31) preserved.

Required for the F.4 integration test to surface R1 in the live stack.
</commit_message>
<xml_diff>
--- a/fixtures/broken_impossible_port_codes.xlsx
+++ b/fixtures/broken_impossible_port_codes.xlsx
@@ -511,7 +511,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ZZZZZ</t>
+          <t>ZZ@ZZ</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -576,7 +576,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>QQQQQ</t>
+          <t>QQ@QQ</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">

</xml_diff>